<commit_message>
Drop the API key, use plain language, fix garbled downloads
- AI help works only in the claude.ai online version with the viewer's own
  Claude account; no API key field or config file. Opened locally, AI
  buttons explain that and everything else works.
- Plain wording across the page, report and Excel via src/labels.js
  (e.g. 必須修改／建議確認／請人工判斷). One large drop zone for the Excel
  workbook; the seven per-file slots move under an "advanced" section.
  Workbook sheets renamed (保單資料、理賠資料、去年保單資料、系統總數);
  old sheet names are still recognised.
- Downloads use ASCII file names (Chinese names could be dropped and saved
  as an extensionless "download"); the issue list downloads as .xlsx, with
  a BOM + CRLF CSV fallback.
- npm run workbook now recalculates formulas with LibreOffice so the
  balance-sheet subtotals are not blank when the file is read.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qz5FvXcAeSpLyKw8NQgMC5
</commit_message>
<xml_diff>
--- a/samples/excel/試用資料_含錯誤.xlsx
+++ b/samples/excel/試用資料_含錯誤.xlsx
@@ -2,28 +2,28 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="說明" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="承保資料" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="給付資料" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="保單資料" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="理賠資料" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="客戶資料" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="商品資料" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="上年度承保資料" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="控制總數" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="去年保單資料" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="系統總數" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="資產負債表" sheetId="8" state="visible" r:id="rId10"/>
     <sheet name="錯誤解答" sheetId="9" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">上年度承保資料!$A$1:$BI$108</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">保單資料!$A$1:$BI$154</definedName>
+    <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">去年保單資料!$A$1:$BI$108</definedName>
     <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">商品資料!$A$1:$G$15</definedName>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">客戶資料!$A$1:$I$240</definedName>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">承保資料!$A$1:$BI$154</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">給付資料!$A$1:$AE$32</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">理賠資料!$A$1:$AE$32</definedName>
     <definedName function="false" hidden="true" localSheetId="8" name="_xlnm._FilterDatabase" vbProcedure="false">錯誤解答!$A$1:$F$73</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19820" uniqueCount="1963">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19820" uniqueCount="1962">
   <si>
     <t xml:space="preserve">申報資料檢核助手｜試用資料（含錯誤）</t>
   </si>
@@ -67,11 +67,11 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">檔整個拖進任一上傳格，工具會依工作表名稱自動分配到各檔案。</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">本檔刻意放入各類錯誤與差異，解答在「錯誤解答」工作表；試用時可先不看解答，比對工具找到的結果。</t>
+      <t xml:space="preserve">檔拖進上方的大框，工具會依工作表名稱自動分好。</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">本檔刻意放入各種錯誤，答案在「錯誤解答」工作表；試用時可先不看答案，比對工具找到的結果。</t>
   </si>
   <si>
     <r>
@@ -80,7 +80,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">欄位：承保／給付／上年度資料的欄位依《人壽保險業個人壽險填報手冊》</t>
+      <t xml:space="preserve">欄位：保單、理賠、去年保單資料的欄位依《人壽保險業個人壽險填報手冊》</t>
     </r>
     <r>
       <rPr>
@@ -114,7 +114,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">；數字欄位以文字儲存，保留前置 </t>
+      <t xml:space="preserve">；數字以文字儲存，保留開頭的 </t>
     </r>
     <r>
       <rPr>
@@ -144,7 +144,7 @@
     <t xml:space="preserve">內容</t>
   </si>
   <si>
-    <t xml:space="preserve">承保資料</t>
+    <t xml:space="preserve">保單資料</t>
   </si>
   <si>
     <r>
@@ -153,7 +153,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">保單資料（承保檔 </t>
+      <t xml:space="preserve">每張保單的申報資料（</t>
     </r>
     <r>
       <rPr>
@@ -162,7 +162,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">LFL</t>
+      <t xml:space="preserve">61 </t>
     </r>
     <r>
       <rPr>
@@ -170,7 +170,20 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">，</t>
+      <t xml:space="preserve">欄）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">理賠資料</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">每筆理賠給付的申報資料（</t>
     </r>
     <r>
       <rPr>
@@ -179,7 +192,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">61 </t>
+      <t xml:space="preserve">31 </t>
     </r>
     <r>
       <rPr>
@@ -191,7 +204,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">給付資料</t>
+    <t xml:space="preserve">客戶資料</t>
   </si>
   <si>
     <r>
@@ -200,7 +213,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">理賠資料（給付檔 </t>
+      <t xml:space="preserve">要保人（角色 </t>
     </r>
     <r>
       <rPr>
@@ -209,7 +222,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">LFD</t>
+      <t xml:space="preserve">1</t>
     </r>
     <r>
       <rPr>
@@ -217,7 +230,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">，</t>
+      <t xml:space="preserve">）與被保險人（角色 </t>
     </r>
     <r>
       <rPr>
@@ -226,7 +239,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">31 </t>
+      <t xml:space="preserve">2</t>
     </r>
     <r>
       <rPr>
@@ -234,11 +247,35 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">欄）</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">客戶資料</t>
+      <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">商品資料</t>
+  </si>
+  <si>
+    <t xml:space="preserve">商品代號、險種、繳費年期、起售日、停售日、替代代號</t>
+  </si>
+  <si>
+    <t xml:space="preserve">去年保單資料</t>
+  </si>
+  <si>
+    <t xml:space="preserve">去年申報的保單資料，用來確認去年底和今年初接得上</t>
+  </si>
+  <si>
+    <t xml:space="preserve">系統總數</t>
+  </si>
+  <si>
+    <t xml:space="preserve">新契約、理賠、保單系統各自的筆數與金額總數，用來核對申報資料</t>
+  </si>
+  <si>
+    <t xml:space="preserve">資產負債表</t>
+  </si>
+  <si>
+    <t xml:space="preserve">各科目餘額，上層科目用公式加總</t>
+  </si>
+  <si>
+    <t xml:space="preserve">錯誤解答</t>
   </si>
   <si>
     <r>
@@ -247,7 +284,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">要保人（角色 </t>
+      <t xml:space="preserve">刻意放入的錯誤和工具應找到的結果（含 </t>
     </r>
     <r>
       <rPr>
@@ -256,7 +293,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1</t>
+      <t xml:space="preserve">4 </t>
     </r>
     <r>
       <rPr>
@@ -264,78 +301,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">）與被保險人（角色 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">）</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">商品資料</t>
-  </si>
-  <si>
-    <t xml:space="preserve">商品代號、險種、繳費年期、起售日、停售日、替代代號</t>
-  </si>
-  <si>
-    <t xml:space="preserve">上年度承保資料</t>
-  </si>
-  <si>
-    <t xml:space="preserve">上年度申報檔，用於期初／期末結轉勾稽</t>
-  </si>
-  <si>
-    <t xml:space="preserve">控制總數</t>
-  </si>
-  <si>
-    <t xml:space="preserve">新契約、理賠、保單管理系統的控制總數，用於跨系統對帳</t>
-  </si>
-  <si>
-    <t xml:space="preserve">資產負債表</t>
-  </si>
-  <si>
-    <t xml:space="preserve">科目餘額（含準備金），上層科目為公式加總</t>
-  </si>
-  <si>
-    <t xml:space="preserve">錯誤解答</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">刻意放入的錯誤與預期的檢核結果（含 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">筆「疑似異常（需人工判斷）」的合理性案例）</t>
+      <t xml:space="preserve">筆「請人工判斷」的不太合理案例）</t>
     </r>
   </si>
   <si>
@@ -433,7 +399,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">注意：承保資料檔中「長度不足」的一筆與「空白行」無法以 </t>
+      <t xml:space="preserve">注意：保單資料文字檔中「長度不足」的一筆與「空白行」無法在 </t>
     </r>
     <r>
       <rPr>
@@ -452,7 +418,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">儲存格表示，請使用 </t>
+      <t xml:space="preserve">中表示，請用 </t>
     </r>
     <r>
       <rPr>
@@ -490,7 +456,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">因此不在本檔「承保資料」，客戶資料會連帶出現 </t>
+      <t xml:space="preserve">因此不在本檔「保單資料」，客戶資料會連帶出現 </t>
     </r>
     <r>
       <rPr>
@@ -12916,7 +12882,7 @@
     <t xml:space="preserve">類別</t>
   </si>
   <si>
-    <t xml:space="preserve">檢核編號</t>
+    <t xml:space="preserve">規則編號</t>
   </si>
   <si>
     <t xml:space="preserve">保單號碼／科目／期間</t>
@@ -12946,7 +12912,7 @@
     <t xml:space="preserve">說明</t>
   </si>
   <si>
-    <t xml:space="preserve">明細檢核</t>
+    <t xml:space="preserve">保單／理賠資料</t>
   </si>
   <si>
     <t xml:space="preserve">23900_L0802</t>
@@ -14556,7 +14522,7 @@
     <t xml:space="preserve">身份為本人，但要保人與被保險人證號不同</t>
   </si>
   <si>
-    <t xml:space="preserve">疑似異常（需人工判斷）</t>
+    <t xml:space="preserve">請人工判斷（不太合理）</t>
   </si>
   <si>
     <t xml:space="preserve">A001</t>
@@ -14605,7 +14571,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">）（不是錯誤：結果應標為疑似異常，由人工判斷）</t>
+      <t xml:space="preserve">）（不算錯誤：工具會標成「請人工判斷」）</t>
     </r>
   </si>
   <si>
@@ -14638,7 +14604,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">（不是錯誤：結果應標為疑似異常，由人工判斷）</t>
+      <t xml:space="preserve">（不算錯誤：工具會標成「請人工判斷」）</t>
     </r>
   </si>
   <si>
@@ -14697,7 +14663,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">）疾病身故（不是錯誤：結果應標為疑似異常，由人工判斷）</t>
+      <t xml:space="preserve">）疾病身故（不算錯誤：工具會標成「請人工判斷」）</t>
     </r>
   </si>
   <si>
@@ -14781,17 +14747,17 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">）身故給付（不是錯誤：結果應標為疑似異常，由人工判斷）</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">匯入規則</t>
+      <t xml:space="preserve">）身故給付（不算錯誤：工具會標成「請人工判斷」）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">自訂規則</t>
   </si>
   <si>
     <t xml:space="preserve">U002</t>
   </si>
   <si>
-    <t xml:space="preserve">承保資料／給付資料</t>
+    <t xml:space="preserve">保單資料／理賠資料</t>
   </si>
   <si>
     <t xml:space="preserve">P250006201/A01</t>
@@ -14820,7 +14786,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">歲承保終身壽險（需先在「規則匯入」套用公司內部核保規則）</t>
+      <t xml:space="preserve">歲承保終身壽險（需先在「新增檢查規則」套用範例的公司內部規則）</t>
     </r>
   </si>
   <si>
@@ -14853,7 +14819,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">萬元未體檢（需先在「規則匯入」套用公司內部核保規則）</t>
+      <t xml:space="preserve">萬元未體檢（需先在「新增檢查規則」套用範例的公司內部規則）</t>
     </r>
   </si>
   <si>
@@ -14886,11 +14852,11 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">天才給付（需先在「規則匯入」套用公司內部核保規則）</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">期初期末結轉</t>
+      <t xml:space="preserve">天才給付（需先在「新增檢查規則」套用範例的公司內部規則）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">去年和今年</t>
   </si>
   <si>
     <t xml:space="preserve">P004</t>
@@ -15027,7 +14993,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">跨系統對帳</t>
+    <t xml:space="preserve">和系統總數比對</t>
   </si>
   <si>
     <t xml:space="preserve">R001</t>
@@ -15068,7 +15034,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">月（應判定為：時間差）</t>
+      <t xml:space="preserve">月（應判定為：結帳日不同）</t>
     </r>
   </si>
   <si>
@@ -15115,7 +15081,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">（應判定為：時間差）</t>
+      <t xml:space="preserve">（應判定為：結帳日不同）</t>
     </r>
   </si>
   <si>
@@ -15188,14 +15154,14 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">（應判定為：時間差）</t>
+      <t xml:space="preserve">（應判定為：結帳日不同）</t>
     </r>
   </si>
   <si>
     <t xml:space="preserve">INF 2025</t>
   </si>
   <si>
-    <t xml:space="preserve">保單管理系統外幣保單以原幣加總（應判定為：定義差）</t>
+    <t xml:space="preserve">保單管理系統外幣保單以原幣加總（應判定為：算法不同）</t>
   </si>
   <si>
     <t xml:space="preserve">NB 2025-03</t>
@@ -15241,11 +15207,8 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">萬元，申報漏報（應判定為：待查）</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">財報勾稽</t>
+      <t xml:space="preserve">萬元，申報漏報（應判定為：需要追查）</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">S008</t>
@@ -15920,7 +15883,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="n">
-        <f aca="false">COUNTA(承保資料!A:A)-1</f>
+        <f aca="false">COUNTA(保單資料!A:A)-1</f>
         <v>153</v>
       </c>
       <c r="C9" s="2" t="s">
@@ -15932,7 +15895,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="2" t="n">
-        <f aca="false">COUNTA(給付資料!A:A)-1</f>
+        <f aca="false">COUNTA(理賠資料!A:A)-1</f>
         <v>31</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -15968,7 +15931,7 @@
         <v>16</v>
       </c>
       <c r="B13" s="2" t="n">
-        <f aca="false">COUNTA(上年度承保資料!A:A)-1</f>
+        <f aca="false">COUNTA(去年保單資料!A:A)-1</f>
         <v>107</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -15980,7 +15943,7 @@
         <v>18</v>
       </c>
       <c r="B14" s="2" t="n">
-        <f aca="false">COUNTA(控制總數!A:A)-1</f>
+        <f aca="false">COUNTA(系統總數!A:A)-1</f>
         <v>26</v>
       </c>
       <c r="C14" s="2" t="s">
@@ -77937,10 +77900,10 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B69" s="10" t="s">
         <v>1952</v>
-      </c>
-      <c r="B69" s="10" t="s">
-        <v>1953</v>
       </c>
       <c r="C69" s="2" t="s">
         <v>20</v>
@@ -77950,15 +77913,15 @@
       </c>
       <c r="E69" s="2"/>
       <c r="F69" s="2" t="s">
-        <v>1954</v>
+        <v>1953</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="s">
-        <v>1952</v>
+        <v>20</v>
       </c>
       <c r="B70" s="10" t="s">
-        <v>1955</v>
+        <v>1954</v>
       </c>
       <c r="C70" s="2" t="s">
         <v>20</v>
@@ -77968,15 +77931,15 @@
       </c>
       <c r="E70" s="2"/>
       <c r="F70" s="2" t="s">
-        <v>1956</v>
+        <v>1955</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2" t="s">
-        <v>1952</v>
+        <v>20</v>
       </c>
       <c r="B71" s="10" t="s">
-        <v>1957</v>
+        <v>1956</v>
       </c>
       <c r="C71" s="2" t="s">
         <v>20</v>
@@ -77986,15 +77949,15 @@
       </c>
       <c r="E71" s="2"/>
       <c r="F71" s="2" t="s">
-        <v>1958</v>
+        <v>1957</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2" t="s">
-        <v>1952</v>
+        <v>20</v>
       </c>
       <c r="B72" s="10" t="s">
-        <v>1959</v>
+        <v>1958</v>
       </c>
       <c r="C72" s="2" t="s">
         <v>20</v>
@@ -78004,15 +77967,15 @@
       </c>
       <c r="E72" s="2"/>
       <c r="F72" s="2" t="s">
-        <v>1960</v>
+        <v>1959</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="2" t="s">
-        <v>1952</v>
+        <v>20</v>
       </c>
       <c r="B73" s="10" t="s">
-        <v>1961</v>
+        <v>1960</v>
       </c>
       <c r="C73" s="2" t="s">
         <v>20</v>
@@ -78022,7 +77985,7 @@
       </c>
       <c r="E73" s="2"/>
       <c r="F73" s="2" t="s">
-        <v>1962</v>
+        <v>1961</v>
       </c>
     </row>
   </sheetData>

</xml_diff>